<commit_message>
replace <Dates>, <States>, <Lgas> to actual values
</commit_message>
<xml_diff>
--- a/api/templates/mtb_detected_rr_detected/en.xlsx
+++ b/api/templates/mtb_detected_rr_detected/en.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>#</t>
   </si>
@@ -61,9 +61,6 @@
     <t>MTB Detected, RR Detected</t>
   </si>
   <si>
-    <t>Dates: &lt;Dates&gt;</t>
-  </si>
-  <si>
     <t>States: &lt;States&gt;</t>
   </si>
   <si>
@@ -99,6 +96,12 @@
   <si>
     <t>Test Notes</t>
   </si>
+  <si>
+    <t>Date Range: &lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t>LGAs: &lt;Lgas&gt;</t>
+  </si>
 </sst>
 </file>
 
@@ -107,12 +110,20 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -200,33 +211,34 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,7 +544,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4990"/>
+  <dimension ref="A1:L4991"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" customWidth="1"/>
@@ -563,8 +575,8 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>15</v>
+      <c r="A2" s="12" t="s">
+        <v>27</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -579,8 +591,8 @@
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>16</v>
+      <c r="A3" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -595,6 +607,9 @@
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>28</v>
+      </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -607,13 +622,8 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2">
-        <v>1</v>
-      </c>
+    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -623,87 +633,102 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
-      <c r="L5" s="4"/>
-    </row>
-    <row r="6" spans="1:12" ht="30.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="4"/>
+    </row>
+    <row r="7" spans="1:12" ht="30.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="D7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="H7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="I7" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="J7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="K7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="L7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+    </row>
+    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L8" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="E8"/>
-    </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E9"/>
     </row>
@@ -15649,6 +15674,9 @@
     </row>
     <row r="4990" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E4990"/>
+    </row>
+    <row r="4991" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E4991"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>